<commit_message>
fix: comprehensive bug fixes - read verification, queue logic, visible browser, pandas import
- Fix missing 'import pandas as pd' in server.py (caused NameError crash)
- Rewrite verify_read: page with content = PASS, only error dialogs = FAIL
- Add _is_error_page() and _page_has_content() shared helpers
- Fix sequential queue: auto-advance to next pending test after completion
- Fix server worker: tc_ids filter BEFORE limit (prevents queue tests being cut off)
- Don't send limit when auto-queue tc_ids are selected
- Keep results table visible after run completes (don't auto-switch to summary)
- Add 'Test Browser (Pop)' button for visible/headed browser debugging
- Update Create/Validate/Setting verifiers to use shared error detection
</commit_message>
<xml_diff>
--- a/automate2/improved/reports/test_results.xlsx
+++ b/automate2/improved/reports/test_results.xlsx
@@ -590,9 +590,9 @@
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Error: Traceback (most recent call last):
-  File "C:\Users\gaykn\Downloads\automate2\improved\webapp\server.py", line 201, in _run_worker
-    status, comment = run_verification(
-                      ^^^^^^^</t>
+  File "C:\Users\gaykn\Downloads\autobom\AUTOMATEBOM\automate2\improved\webapp\server.py", line 238, in _run_worker
+    _state["total"] = total
+    _broadcast("</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-10 19:13</t>
+          <t>2026-08-10 21:29</t>
         </is>
       </c>
     </row>

</xml_diff>